<commit_message>
small additions/changes to incorrect data
</commit_message>
<xml_diff>
--- a/Iteration 2/Agile Gantt chart .xlsx
+++ b/Iteration 2/Agile Gantt chart .xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="854" documentId="8_{5FCFFA2A-1C94-4F30-8EBC-885A9A0A3AE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B23A52CC-7651-4A1E-92EA-292508F0024C}"/>
+  <xr:revisionPtr revIDLastSave="916" documentId="8_{5FCFFA2A-1C94-4F30-8EBC-885A9A0A3AE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA54B23A-657F-48AB-B515-C65E66D4E772}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" tabRatio="415" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="83">
   <si>
     <t>Task 3</t>
   </si>
@@ -306,6 +306,9 @@
   </si>
   <si>
     <t>BREAK</t>
+  </si>
+  <si>
+    <t>Complete all tasks for Iteration 2 and submit Progress Reports</t>
   </si>
 </sst>
 </file>
@@ -932,7 +935,7 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="146">
+  <cellXfs count="147">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1270,6 +1273,18 @@
     <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1321,16 +1336,7 @@
     <xf numFmtId="0" fontId="10" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2641,6 +2647,75 @@
       </border>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-9.9948118533890809E-2"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
       <font>
         <color auto="1"/>
       </font>
@@ -2768,75 +2843,6 @@
       </border>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-9.9948118533890809E-2"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -2890,121 +2896,6 @@
           <color theme="0" tint="-0.34998626667073579"/>
         </bottom>
       </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" relativeIndent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1" tint="0.249977111117893"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -3170,6 +3061,121 @@
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1" tint="0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" relativeIndent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
       </font>
     </dxf>
     <dxf>
@@ -3587,7 +3593,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp1.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Scroll" dx="39" fmlaLink="$C$7" horiz="1" max="365" page="2" val="24"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Scroll" dx="39" fmlaLink="$C$7" horiz="1" max="365" page="2" val="0"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3689,7 +3695,7 @@
                   <a14:compatExt spid="_x0000_s24577"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F667727B-F99A-4D52-8073-58F3A4893BD7}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000001600000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -3744,7 +3750,7 @@
                   <a14:compatExt spid="_x0000_s19457"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-0000014C0000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-0000014C0000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -3799,7 +3805,7 @@
                   <a14:compatExt spid="_x0000_s16385"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000001400000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000001400000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -3854,7 +3860,7 @@
                   <a14:compatExt spid="_x0000_s13313"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000001340000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000001340000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -3909,7 +3915,7 @@
                   <a14:compatExt spid="_x0000_s17409"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000001440000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-000001440000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -3944,8 +3950,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A9DCD786-338F-4F4D-899D-936CC39D523A}" name="Milestones435263" displayName="Milestones435263" ref="B9:G38" totalsRowShown="0" headerRowDxfId="98" dataDxfId="97">
-  <autoFilter ref="B9:G38" xr:uid="{29E5A880-80D5-4B65-B5FB-8FB3913D3D27}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A9DCD786-338F-4F4D-899D-936CC39D523A}" name="Milestones435263" displayName="Milestones435263" ref="B9:G41" totalsRowShown="0" headerRowDxfId="126" dataDxfId="125">
+  <autoFilter ref="B9:G41" xr:uid="{29E5A880-80D5-4B65-B5FB-8FB3913D3D27}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -3954,12 +3960,12 @@
     <filterColumn colId="5" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{40445EDE-9593-4FF7-8BAE-92234704569C}" name="Milestone description" dataDxfId="96"/>
-    <tableColumn id="2" xr3:uid="{68BCB8EB-CD74-458C-BC89-842312A712BF}" name="Category" dataDxfId="95"/>
-    <tableColumn id="3" xr3:uid="{E5449758-B90F-41ED-8762-83300E9616BD}" name="Assigned to" dataDxfId="94"/>
-    <tableColumn id="4" xr3:uid="{0C1E43FF-25F9-4BA6-B852-4E28BC5D9427}" name="Progress" dataDxfId="93"/>
-    <tableColumn id="5" xr3:uid="{78F71E7D-C2CE-4D9A-AD17-E5A1BEC14C24}" name="Start" dataDxfId="92" dataCellStyle="Date"/>
-    <tableColumn id="6" xr3:uid="{05DEF285-72DF-4ADA-BA39-0ED70BDDA00E}" name="Days" dataDxfId="91" dataCellStyle="Comma [0]"/>
+    <tableColumn id="1" xr3:uid="{40445EDE-9593-4FF7-8BAE-92234704569C}" name="Milestone description" dataDxfId="124"/>
+    <tableColumn id="2" xr3:uid="{68BCB8EB-CD74-458C-BC89-842312A712BF}" name="Category" dataDxfId="123"/>
+    <tableColumn id="3" xr3:uid="{E5449758-B90F-41ED-8762-83300E9616BD}" name="Assigned to" dataDxfId="122"/>
+    <tableColumn id="4" xr3:uid="{0C1E43FF-25F9-4BA6-B852-4E28BC5D9427}" name="Progress" dataDxfId="121"/>
+    <tableColumn id="5" xr3:uid="{78F71E7D-C2CE-4D9A-AD17-E5A1BEC14C24}" name="Start" dataDxfId="120" dataCellStyle="Date"/>
+    <tableColumn id="6" xr3:uid="{05DEF285-72DF-4ADA-BA39-0ED70BDDA00E}" name="Days" dataDxfId="119" dataCellStyle="Comma [0]"/>
   </tableColumns>
   <tableStyleInfo name="ToDoList" showFirstColumn="1" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
@@ -3971,7 +3977,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{BE3B58B4-F4CD-42FF-AF8A-57DABD72004E}" name="Milestones43526" displayName="Milestones43526" ref="B9:G36" totalsRowShown="0" headerRowDxfId="126" dataDxfId="125">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{BE3B58B4-F4CD-42FF-AF8A-57DABD72004E}" name="Milestones43526" displayName="Milestones43526" ref="B9:G36" totalsRowShown="0" headerRowDxfId="118" dataDxfId="117">
   <autoFilter ref="B9:G36" xr:uid="{29E5A880-80D5-4B65-B5FB-8FB3913D3D27}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -3981,12 +3987,12 @@
     <filterColumn colId="5" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{672FF862-0C07-4252-9134-1252089DA775}" name="Milestone description" dataDxfId="124"/>
-    <tableColumn id="2" xr3:uid="{48A09342-46E9-4A90-B54C-3424B55EC3D1}" name="Category" dataDxfId="123"/>
-    <tableColumn id="3" xr3:uid="{B605E6EA-8F40-4F08-9A6C-D7CF67247964}" name="Assigned to" dataDxfId="122"/>
-    <tableColumn id="4" xr3:uid="{DA0732FA-EAE6-4606-B4E6-47DB2A2B9562}" name="Progress" dataDxfId="121"/>
-    <tableColumn id="5" xr3:uid="{21DD67FA-45E1-4867-8807-A05E83F9636C}" name="Start" dataDxfId="120" dataCellStyle="Date"/>
-    <tableColumn id="6" xr3:uid="{C9828D43-9B77-44CB-89EC-F1B963F6A043}" name="Days" dataDxfId="119" dataCellStyle="Comma [0]"/>
+    <tableColumn id="1" xr3:uid="{672FF862-0C07-4252-9134-1252089DA775}" name="Milestone description" dataDxfId="116"/>
+    <tableColumn id="2" xr3:uid="{48A09342-46E9-4A90-B54C-3424B55EC3D1}" name="Category" dataDxfId="115"/>
+    <tableColumn id="3" xr3:uid="{B605E6EA-8F40-4F08-9A6C-D7CF67247964}" name="Assigned to" dataDxfId="114"/>
+    <tableColumn id="4" xr3:uid="{DA0732FA-EAE6-4606-B4E6-47DB2A2B9562}" name="Progress" dataDxfId="113"/>
+    <tableColumn id="5" xr3:uid="{21DD67FA-45E1-4867-8807-A05E83F9636C}" name="Start" dataDxfId="112" dataCellStyle="Date"/>
+    <tableColumn id="6" xr3:uid="{C9828D43-9B77-44CB-89EC-F1B963F6A043}" name="Days" dataDxfId="111" dataCellStyle="Comma [0]"/>
   </tableColumns>
   <tableStyleInfo name="ToDoList" showFirstColumn="1" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
@@ -3998,7 +4004,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DD82988E-1813-40AE-BDE7-9F0200A703CB}" name="Milestones4352" displayName="Milestones4352" ref="B9:G36" totalsRowShown="0" headerRowDxfId="118" dataDxfId="117">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DD82988E-1813-40AE-BDE7-9F0200A703CB}" name="Milestones4352" displayName="Milestones4352" ref="B9:G36" totalsRowShown="0" headerRowDxfId="110" dataDxfId="109">
   <autoFilter ref="B9:G36" xr:uid="{29E5A880-80D5-4B65-B5FB-8FB3913D3D27}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4008,12 +4014,12 @@
     <filterColumn colId="5" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{619BF8F6-D0F1-41AD-871D-FE0240C45A93}" name="Milestone description" dataDxfId="116"/>
-    <tableColumn id="2" xr3:uid="{39BD914E-FB02-4352-846C-6D59624DC0B0}" name="Category" dataDxfId="115"/>
-    <tableColumn id="3" xr3:uid="{D274194F-BCA0-44F3-84B2-217254EE241C}" name="Assigned to" dataDxfId="114"/>
-    <tableColumn id="4" xr3:uid="{8385BC6F-56EE-4363-A106-8DB0A1E4EF5A}" name="Progress" dataDxfId="113"/>
-    <tableColumn id="5" xr3:uid="{02926609-7B93-4B6F-BE96-92EC7A949E4B}" name="Start" dataDxfId="112" dataCellStyle="Date"/>
-    <tableColumn id="6" xr3:uid="{8FF9BE8E-04B7-4B39-AC27-D2E534204BC3}" name="Days" dataDxfId="111" dataCellStyle="Comma [0]"/>
+    <tableColumn id="1" xr3:uid="{619BF8F6-D0F1-41AD-871D-FE0240C45A93}" name="Milestone description" dataDxfId="108"/>
+    <tableColumn id="2" xr3:uid="{39BD914E-FB02-4352-846C-6D59624DC0B0}" name="Category" dataDxfId="107"/>
+    <tableColumn id="3" xr3:uid="{D274194F-BCA0-44F3-84B2-217254EE241C}" name="Assigned to" dataDxfId="106"/>
+    <tableColumn id="4" xr3:uid="{8385BC6F-56EE-4363-A106-8DB0A1E4EF5A}" name="Progress" dataDxfId="105"/>
+    <tableColumn id="5" xr3:uid="{02926609-7B93-4B6F-BE96-92EC7A949E4B}" name="Start" dataDxfId="104" dataCellStyle="Date"/>
+    <tableColumn id="6" xr3:uid="{8FF9BE8E-04B7-4B39-AC27-D2E534204BC3}" name="Days" dataDxfId="103" dataCellStyle="Comma [0]"/>
   </tableColumns>
   <tableStyleInfo name="ToDoList" showFirstColumn="1" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
@@ -4025,7 +4031,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0EDB95CA-98FE-4198-8801-690B9B480FDF}" name="Milestones435" displayName="Milestones435" ref="B9:G43" totalsRowShown="0" headerRowDxfId="110" dataDxfId="109">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0EDB95CA-98FE-4198-8801-690B9B480FDF}" name="Milestones435" displayName="Milestones435" ref="B9:G43" totalsRowShown="0" headerRowDxfId="102" dataDxfId="101">
   <autoFilter ref="B9:G43" xr:uid="{29E5A880-80D5-4B65-B5FB-8FB3913D3D27}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4035,12 +4041,12 @@
     <filterColumn colId="5" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{6E47A83D-ACD7-4EB6-9B84-5195E813945E}" name="Milestone description" dataDxfId="108"/>
-    <tableColumn id="2" xr3:uid="{529EEF64-D037-4ACF-8CA4-0C10FE2D1FBB}" name="Category" dataDxfId="107"/>
-    <tableColumn id="3" xr3:uid="{711D01BA-2785-403A-9636-CCC7E2ADA584}" name="Assigned to" dataDxfId="106"/>
-    <tableColumn id="4" xr3:uid="{62B00BEF-16BE-4692-B5E2-F287F680F2C1}" name="Progress" dataDxfId="105"/>
-    <tableColumn id="5" xr3:uid="{D6D72902-F68F-4E59-A714-AFFF520C647A}" name="Start" dataDxfId="104" dataCellStyle="Date"/>
-    <tableColumn id="6" xr3:uid="{93E698DE-286F-49ED-AA20-D0C843671DE8}" name="Days" dataDxfId="103" dataCellStyle="Comma [0]"/>
+    <tableColumn id="1" xr3:uid="{6E47A83D-ACD7-4EB6-9B84-5195E813945E}" name="Milestone description" dataDxfId="100"/>
+    <tableColumn id="2" xr3:uid="{529EEF64-D037-4ACF-8CA4-0C10FE2D1FBB}" name="Category" dataDxfId="99"/>
+    <tableColumn id="3" xr3:uid="{711D01BA-2785-403A-9636-CCC7E2ADA584}" name="Assigned to" dataDxfId="98"/>
+    <tableColumn id="4" xr3:uid="{62B00BEF-16BE-4692-B5E2-F287F680F2C1}" name="Progress" dataDxfId="97"/>
+    <tableColumn id="5" xr3:uid="{D6D72902-F68F-4E59-A714-AFFF520C647A}" name="Start" dataDxfId="96" dataCellStyle="Date"/>
+    <tableColumn id="6" xr3:uid="{93E698DE-286F-49ED-AA20-D0C843671DE8}" name="Days" dataDxfId="95" dataCellStyle="Comma [0]"/>
   </tableColumns>
   <tableStyleInfo name="Gantt Table Style" showFirstColumn="1" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
@@ -4052,7 +4058,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{876EA49D-634E-482B-8173-880F7B761E2C}" name="Milestones43524" displayName="Milestones43524" ref="B9:G36" totalsRowShown="0" headerRowDxfId="102">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{876EA49D-634E-482B-8173-880F7B761E2C}" name="Milestones43524" displayName="Milestones43524" ref="B9:G36" totalsRowShown="0" headerRowDxfId="94">
   <autoFilter ref="B9:G36" xr:uid="{29E5A880-80D5-4B65-B5FB-8FB3913D3D27}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4062,9 +4068,9 @@
     <filterColumn colId="5" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{0971B905-713A-4980-8BBC-DF959C2E61F9}" name="Milestone description" dataDxfId="101"/>
-    <tableColumn id="2" xr3:uid="{4492A0B8-068F-4002-9E8D-E1F5FED367F0}" name="Category" dataDxfId="100"/>
-    <tableColumn id="3" xr3:uid="{DF1A764E-7050-4528-B7F9-B6AB99372146}" name="Assigned to" dataDxfId="99"/>
+    <tableColumn id="1" xr3:uid="{0971B905-713A-4980-8BBC-DF959C2E61F9}" name="Milestone description" dataDxfId="93"/>
+    <tableColumn id="2" xr3:uid="{4492A0B8-068F-4002-9E8D-E1F5FED367F0}" name="Category" dataDxfId="92"/>
+    <tableColumn id="3" xr3:uid="{DF1A764E-7050-4528-B7F9-B6AB99372146}" name="Assigned to" dataDxfId="91"/>
     <tableColumn id="4" xr3:uid="{47C54592-75B0-4C70-BBF8-0F40483670E9}" name="Progress"/>
     <tableColumn id="5" xr3:uid="{663FB5E0-7616-4EA5-B56A-FF069E2E07D7}" name="Start" dataCellStyle="Date"/>
     <tableColumn id="6" xr3:uid="{3B766962-C06F-4E12-BE91-12AB93439874}" name="Days" dataCellStyle="Comma [0]"/>
@@ -4358,11 +4364,11 @@
     <row r="2" spans="1:13" ht="50.15" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A2" s="7"/>
       <c r="B2" s="107"/>
-      <c r="C2" s="133" t="s">
+      <c r="C2" s="137" t="s">
         <v>32</v>
       </c>
-      <c r="D2" s="133"/>
-      <c r="E2" s="133"/>
+      <c r="D2" s="137"/>
+      <c r="E2" s="137"/>
       <c r="F2" s="107"/>
       <c r="G2" s="7"/>
       <c r="H2" s="7"/>
@@ -4390,11 +4396,11 @@
     <row r="4" spans="1:13" s="8" customFormat="1" ht="67.150000000000006" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A4" s="7"/>
       <c r="B4" s="102"/>
-      <c r="C4" s="134" t="s">
+      <c r="C4" s="138" t="s">
         <v>33</v>
       </c>
-      <c r="D4" s="134"/>
-      <c r="E4" s="134"/>
+      <c r="D4" s="138"/>
+      <c r="E4" s="138"/>
       <c r="F4" s="102"/>
       <c r="G4" s="7"/>
       <c r="H4" s="7"/>
@@ -4407,11 +4413,11 @@
     <row r="5" spans="1:13" s="8" customFormat="1" ht="67.150000000000006" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A5" s="7"/>
       <c r="B5" s="102"/>
-      <c r="C5" s="134" t="s">
+      <c r="C5" s="138" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="134"/>
-      <c r="E5" s="134"/>
+      <c r="D5" s="138"/>
+      <c r="E5" s="138"/>
       <c r="F5" s="102"/>
       <c r="G5" s="7"/>
       <c r="H5" s="7"/>
@@ -4511,7 +4517,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BP40"/>
+  <dimension ref="A1:BP43"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4.7265625" style="9" customWidth="1"/>
@@ -4529,27 +4535,27 @@
     <row r="1" spans="1:68" ht="25.15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="1:68" ht="49.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="10"/>
-      <c r="B2" s="127" t="s">
+      <c r="B2" s="131" t="s">
         <v>73</v>
       </c>
-      <c r="C2" s="127"/>
-      <c r="D2" s="127"/>
-      <c r="E2" s="127"/>
-      <c r="F2" s="127"/>
-      <c r="G2" s="127"/>
-      <c r="H2" s="127"/>
-      <c r="I2" s="128"/>
-      <c r="J2" s="128"/>
-      <c r="K2" s="128"/>
-      <c r="L2" s="128"/>
-      <c r="M2" s="128"/>
-      <c r="N2" s="128"/>
-      <c r="O2" s="129"/>
-      <c r="P2" s="129"/>
-      <c r="Q2" s="129"/>
-      <c r="R2" s="129"/>
-      <c r="S2" s="129"/>
-      <c r="T2" s="129"/>
+      <c r="C2" s="131"/>
+      <c r="D2" s="131"/>
+      <c r="E2" s="131"/>
+      <c r="F2" s="131"/>
+      <c r="G2" s="131"/>
+      <c r="H2" s="131"/>
+      <c r="I2" s="132"/>
+      <c r="J2" s="132"/>
+      <c r="K2" s="132"/>
+      <c r="L2" s="132"/>
+      <c r="M2" s="132"/>
+      <c r="N2" s="132"/>
+      <c r="O2" s="133"/>
+      <c r="P2" s="133"/>
+      <c r="Q2" s="133"/>
+      <c r="R2" s="133"/>
+      <c r="S2" s="133"/>
+      <c r="T2" s="133"/>
       <c r="U2" s="61"/>
       <c r="V2" s="61"/>
       <c r="W2" s="61"/>
@@ -4623,36 +4629,36 @@
         <v>18</v>
       </c>
       <c r="H4" s="69"/>
-      <c r="I4" s="130" t="s">
+      <c r="I4" s="134" t="s">
         <v>25</v>
       </c>
-      <c r="J4" s="130"/>
-      <c r="K4" s="130"/>
-      <c r="L4" s="130"/>
-      <c r="N4" s="131" t="s">
+      <c r="J4" s="134"/>
+      <c r="K4" s="134"/>
+      <c r="L4" s="134"/>
+      <c r="N4" s="135" t="s">
         <v>26</v>
       </c>
-      <c r="O4" s="131"/>
-      <c r="P4" s="131"/>
-      <c r="Q4" s="131"/>
-      <c r="S4" s="132" t="s">
+      <c r="O4" s="135"/>
+      <c r="P4" s="135"/>
+      <c r="Q4" s="135"/>
+      <c r="S4" s="136" t="s">
         <v>27</v>
       </c>
-      <c r="T4" s="132"/>
-      <c r="U4" s="132"/>
-      <c r="V4" s="132"/>
-      <c r="X4" s="125" t="s">
+      <c r="T4" s="136"/>
+      <c r="U4" s="136"/>
+      <c r="V4" s="136"/>
+      <c r="X4" s="129" t="s">
         <v>28</v>
       </c>
-      <c r="Y4" s="125"/>
-      <c r="Z4" s="125"/>
-      <c r="AA4" s="125"/>
-      <c r="AC4" s="126" t="s">
+      <c r="Y4" s="129"/>
+      <c r="Z4" s="129"/>
+      <c r="AA4" s="129"/>
+      <c r="AC4" s="130" t="s">
         <v>19</v>
       </c>
-      <c r="AD4" s="126"/>
-      <c r="AE4" s="126"/>
-      <c r="AF4" s="126"/>
+      <c r="AD4" s="130"/>
+      <c r="AE4" s="130"/>
+      <c r="AF4" s="130"/>
     </row>
     <row r="5" spans="1:68" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="10"/>
@@ -4681,7 +4687,7 @@
       <c r="H6" s="69"/>
       <c r="I6" s="85" t="str">
         <f ca="1">TEXT(I7,"mmmm")</f>
-        <v>March</v>
+        <v>February</v>
       </c>
       <c r="J6" s="85"/>
       <c r="K6" s="85"/>
@@ -4691,7 +4697,7 @@
       <c r="O6" s="85"/>
       <c r="P6" s="85" t="str">
         <f ca="1">IF(TEXT(P7,"mmmm")=I6,"",TEXT(P7,"mmmm"))</f>
-        <v/>
+        <v>March</v>
       </c>
       <c r="Q6" s="85"/>
       <c r="R6" s="85"/>
@@ -4701,7 +4707,7 @@
       <c r="V6" s="85"/>
       <c r="W6" s="85" t="str">
         <f ca="1">IF(OR(TEXT(W7,"mmmm")=P6,TEXT(W7,"mmmm")=I6),"",TEXT(W7,"mmmm"))</f>
-        <v>April</v>
+        <v/>
       </c>
       <c r="X6" s="85"/>
       <c r="Y6" s="85"/>
@@ -4731,7 +4737,7 @@
       <c r="AQ6" s="85"/>
       <c r="AR6" s="85" t="str">
         <f ca="1">IF(OR(TEXT(AR7,"mmmm")=AK6,TEXT(AR7,"mmmm")=AD6,TEXT(AR7,"mmmm")=W6,TEXT(AR7,"mmmm")=P6),"",TEXT(AR7,"mmmm"))</f>
-        <v/>
+        <v>April</v>
       </c>
       <c r="AS6" s="85"/>
       <c r="AT6" s="85"/>
@@ -4741,7 +4747,7 @@
       <c r="AX6" s="86"/>
       <c r="AY6" s="86" t="str">
         <f ca="1">IF(OR(TEXT(AY7,"mmmm")=AR6,TEXT(AY7,"mmmm")=AK6,TEXT(AY7,"mmmm")=AD6,TEXT(AY7,"mmmm")=W6),"",TEXT(AY7,"mmmm"))</f>
-        <v>May</v>
+        <v/>
       </c>
       <c r="AZ6" s="86"/>
       <c r="BA6" s="86"/>
@@ -4766,7 +4772,7 @@
         <v>12</v>
       </c>
       <c r="C7" s="76">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="D7" s="68"/>
       <c r="E7" s="69"/>
@@ -4775,227 +4781,227 @@
       <c r="H7" s="77"/>
       <c r="I7" s="92">
         <f ca="1">IFERROR(Project_Start+Scrolling_Increment,TODAY())</f>
-        <v>46102</v>
+        <v>46078</v>
       </c>
       <c r="J7" s="93">
         <f ca="1">I7+1</f>
-        <v>46103</v>
+        <v>46079</v>
       </c>
       <c r="K7" s="93">
         <f t="shared" ref="K7:AX7" ca="1" si="0">J7+1</f>
-        <v>46104</v>
+        <v>46080</v>
       </c>
       <c r="L7" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>46105</v>
+        <v>46081</v>
       </c>
       <c r="M7" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>46106</v>
+        <v>46082</v>
       </c>
       <c r="N7" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>46107</v>
+        <v>46083</v>
       </c>
       <c r="O7" s="94">
         <f t="shared" ca="1" si="0"/>
-        <v>46108</v>
+        <v>46084</v>
       </c>
       <c r="P7" s="93">
         <f ca="1">O7+1</f>
-        <v>46109</v>
+        <v>46085</v>
       </c>
       <c r="Q7" s="93">
         <f ca="1">P7+1</f>
-        <v>46110</v>
+        <v>46086</v>
       </c>
       <c r="R7" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>46111</v>
+        <v>46087</v>
       </c>
       <c r="S7" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>46112</v>
+        <v>46088</v>
       </c>
       <c r="T7" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>46113</v>
+        <v>46089</v>
       </c>
       <c r="U7" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>46114</v>
+        <v>46090</v>
       </c>
       <c r="V7" s="94">
         <f t="shared" ca="1" si="0"/>
-        <v>46115</v>
+        <v>46091</v>
       </c>
       <c r="W7" s="93">
         <f ca="1">V7+1</f>
-        <v>46116</v>
+        <v>46092</v>
       </c>
       <c r="X7" s="93">
         <f ca="1">W7+1</f>
-        <v>46117</v>
+        <v>46093</v>
       </c>
       <c r="Y7" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>46118</v>
+        <v>46094</v>
       </c>
       <c r="Z7" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>46119</v>
+        <v>46095</v>
       </c>
       <c r="AA7" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>46120</v>
+        <v>46096</v>
       </c>
       <c r="AB7" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>46121</v>
+        <v>46097</v>
       </c>
       <c r="AC7" s="94">
         <f t="shared" ca="1" si="0"/>
-        <v>46122</v>
+        <v>46098</v>
       </c>
       <c r="AD7" s="93">
         <f ca="1">AC7+1</f>
-        <v>46123</v>
+        <v>46099</v>
       </c>
       <c r="AE7" s="93">
         <f ca="1">AD7+1</f>
-        <v>46124</v>
+        <v>46100</v>
       </c>
       <c r="AF7" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>46125</v>
+        <v>46101</v>
       </c>
       <c r="AG7" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>46126</v>
+        <v>46102</v>
       </c>
       <c r="AH7" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>46127</v>
+        <v>46103</v>
       </c>
       <c r="AI7" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>46128</v>
+        <v>46104</v>
       </c>
       <c r="AJ7" s="94">
         <f t="shared" ca="1" si="0"/>
-        <v>46129</v>
+        <v>46105</v>
       </c>
       <c r="AK7" s="93">
         <f ca="1">AJ7+1</f>
-        <v>46130</v>
+        <v>46106</v>
       </c>
       <c r="AL7" s="93">
         <f ca="1">AK7+1</f>
-        <v>46131</v>
+        <v>46107</v>
       </c>
       <c r="AM7" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>46132</v>
+        <v>46108</v>
       </c>
       <c r="AN7" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>46133</v>
+        <v>46109</v>
       </c>
       <c r="AO7" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>46134</v>
+        <v>46110</v>
       </c>
       <c r="AP7" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>46135</v>
+        <v>46111</v>
       </c>
       <c r="AQ7" s="94">
         <f t="shared" ca="1" si="0"/>
-        <v>46136</v>
+        <v>46112</v>
       </c>
       <c r="AR7" s="93">
         <f ca="1">AQ7+1</f>
-        <v>46137</v>
+        <v>46113</v>
       </c>
       <c r="AS7" s="93">
         <f ca="1">AR7+1</f>
-        <v>46138</v>
+        <v>46114</v>
       </c>
       <c r="AT7" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>46139</v>
+        <v>46115</v>
       </c>
       <c r="AU7" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>46140</v>
+        <v>46116</v>
       </c>
       <c r="AV7" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>46141</v>
+        <v>46117</v>
       </c>
       <c r="AW7" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>46142</v>
+        <v>46118</v>
       </c>
       <c r="AX7" s="94">
         <f t="shared" ca="1" si="0"/>
-        <v>46143</v>
+        <v>46119</v>
       </c>
       <c r="AY7" s="93">
         <f ca="1">AX7+1</f>
-        <v>46144</v>
+        <v>46120</v>
       </c>
       <c r="AZ7" s="93">
         <f ca="1">AY7+1</f>
-        <v>46145</v>
+        <v>46121</v>
       </c>
       <c r="BA7" s="93">
         <f t="shared" ref="BA7:BE7" ca="1" si="1">AZ7+1</f>
-        <v>46146</v>
+        <v>46122</v>
       </c>
       <c r="BB7" s="93">
         <f t="shared" ca="1" si="1"/>
-        <v>46147</v>
+        <v>46123</v>
       </c>
       <c r="BC7" s="93">
         <f t="shared" ca="1" si="1"/>
-        <v>46148</v>
+        <v>46124</v>
       </c>
       <c r="BD7" s="93">
         <f t="shared" ca="1" si="1"/>
-        <v>46149</v>
+        <v>46125</v>
       </c>
       <c r="BE7" s="94">
         <f t="shared" ca="1" si="1"/>
-        <v>46150</v>
+        <v>46126</v>
       </c>
       <c r="BF7" s="93">
         <f ca="1">BE7+1</f>
-        <v>46151</v>
+        <v>46127</v>
       </c>
       <c r="BG7" s="93">
         <f ca="1">BF7+1</f>
-        <v>46152</v>
+        <v>46128</v>
       </c>
       <c r="BH7" s="93">
         <f t="shared" ref="BH7:BL7" ca="1" si="2">BG7+1</f>
-        <v>46153</v>
+        <v>46129</v>
       </c>
       <c r="BI7" s="93">
         <f t="shared" ca="1" si="2"/>
-        <v>46154</v>
+        <v>46130</v>
       </c>
       <c r="BJ7" s="93">
         <f t="shared" ca="1" si="2"/>
-        <v>46155</v>
+        <v>46131</v>
       </c>
       <c r="BK7" s="93">
         <f t="shared" ca="1" si="2"/>
-        <v>46156</v>
+        <v>46132</v>
       </c>
       <c r="BL7" s="94">
         <f t="shared" ca="1" si="2"/>
-        <v>46157</v>
+        <v>46133</v>
       </c>
     </row>
     <row r="8" spans="1:68" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -5087,227 +5093,227 @@
       <c r="H9" s="82"/>
       <c r="I9" s="100" t="str">
         <f t="shared" ref="I9:BL9" ca="1" si="3">LEFT(TEXT(I7,"ddd"),1)</f>
-        <v>S</v>
+        <v>W</v>
       </c>
       <c r="J9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>T</v>
       </c>
       <c r="K9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>F</v>
       </c>
       <c r="L9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>S</v>
       </c>
       <c r="M9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>S</v>
       </c>
       <c r="N9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>M</v>
       </c>
       <c r="O9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>T</v>
       </c>
       <c r="P9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>W</v>
       </c>
       <c r="Q9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>T</v>
       </c>
       <c r="R9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>F</v>
       </c>
       <c r="S9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>S</v>
       </c>
       <c r="T9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>S</v>
       </c>
       <c r="U9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>M</v>
       </c>
       <c r="V9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>T</v>
       </c>
       <c r="W9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>W</v>
       </c>
       <c r="X9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>T</v>
       </c>
       <c r="Y9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>F</v>
       </c>
       <c r="Z9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>S</v>
       </c>
       <c r="AA9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>S</v>
       </c>
       <c r="AB9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>M</v>
       </c>
       <c r="AC9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>T</v>
       </c>
       <c r="AD9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>W</v>
       </c>
       <c r="AE9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>T</v>
       </c>
       <c r="AF9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>F</v>
       </c>
       <c r="AG9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>S</v>
       </c>
       <c r="AH9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>S</v>
       </c>
       <c r="AI9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>M</v>
       </c>
       <c r="AJ9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>T</v>
       </c>
       <c r="AK9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>W</v>
       </c>
       <c r="AL9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>T</v>
       </c>
       <c r="AM9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>F</v>
       </c>
       <c r="AN9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>S</v>
       </c>
       <c r="AO9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>S</v>
       </c>
       <c r="AP9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>M</v>
       </c>
       <c r="AQ9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>T</v>
       </c>
       <c r="AR9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>W</v>
       </c>
       <c r="AS9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>T</v>
       </c>
       <c r="AT9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>F</v>
       </c>
       <c r="AU9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>S</v>
       </c>
       <c r="AV9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>S</v>
       </c>
       <c r="AW9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>M</v>
       </c>
       <c r="AX9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>T</v>
       </c>
       <c r="AY9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>W</v>
       </c>
       <c r="AZ9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>T</v>
       </c>
       <c r="BA9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>F</v>
       </c>
       <c r="BB9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>S</v>
       </c>
       <c r="BC9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>S</v>
       </c>
       <c r="BD9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>M</v>
       </c>
       <c r="BE9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>T</v>
       </c>
       <c r="BF9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>W</v>
       </c>
       <c r="BG9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>T</v>
       </c>
       <c r="BH9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>F</v>
       </c>
       <c r="BI9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>S</v>
       </c>
       <c r="BJ9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>S</v>
       </c>
       <c r="BK9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>M</v>
       </c>
       <c r="BL9" s="100" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>T</v>
       </c>
     </row>
     <row r="10" spans="1:68" ht="30" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5632,9 +5638,9 @@
         <v>1</v>
       </c>
       <c r="H12" s="53"/>
-      <c r="I12" s="22" t="str">
+      <c r="I12" s="22">
         <f ca="1">IF(AND($C12="Goal",I$7&gt;=$F12,I$7&lt;=$F12+$G12-1),2,IF(AND($C12="Milestone",I$7&gt;=$F12,I$7&lt;=$F12+$G12-1),1,""))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="J12" s="22" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -5859,7 +5865,7 @@
     </row>
     <row r="13" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="10"/>
-      <c r="B13" s="142" t="s">
+      <c r="B13" s="125" t="s">
         <v>75</v>
       </c>
       <c r="C13" s="81" t="s">
@@ -5878,9 +5884,9 @@
         <v>1</v>
       </c>
       <c r="H13" s="53"/>
-      <c r="I13" s="22" t="str">
+      <c r="I13" s="22">
         <f t="shared" ref="I13:X28" ca="1" si="8">IF(AND($C13="Goal",I$7&gt;=$F13,I$7&lt;=$F13+$G13-1),2,IF(AND($C13="Milestone",I$7&gt;=$F13,I$7&lt;=$F13+$G13-1),1,""))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="J13" s="22" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -6112,7 +6118,7 @@
         <v>16</v>
       </c>
       <c r="D14" s="81" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="E14" s="54">
         <v>1</v>
@@ -6351,7 +6357,7 @@
     </row>
     <row r="15" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="9"/>
-      <c r="B15" s="142" t="s">
+      <c r="B15" s="125" t="s">
         <v>76</v>
       </c>
       <c r="C15" s="81" t="s">
@@ -6398,9 +6404,9 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-      <c r="P15" s="22" t="str">
-        <f t="shared" ca="1" si="4"/>
-        <v/>
+      <c r="P15" s="22">
+        <f t="shared" ca="1" si="4"/>
+        <v>2</v>
       </c>
       <c r="Q15" s="22" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -6843,7 +6849,7 @@
     </row>
     <row r="17" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="10"/>
-      <c r="B17" s="142" t="s">
+      <c r="B17" s="125" t="s">
         <v>77</v>
       </c>
       <c r="C17" s="81" t="s">
@@ -6914,9 +6920,9 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-      <c r="V17" s="22" t="str">
-        <f t="shared" ca="1" si="4"/>
-        <v/>
+      <c r="V17" s="22">
+        <f t="shared" ca="1" si="4"/>
+        <v>2</v>
       </c>
       <c r="W17" s="22" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -7342,7 +7348,7 @@
         <v>16</v>
       </c>
       <c r="D19" s="81" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E19" s="54">
         <v>1</v>
@@ -7827,7 +7833,7 @@
     </row>
     <row r="21" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="9"/>
-      <c r="B21" s="142" t="s">
+      <c r="B21" s="125" t="s">
         <v>78</v>
       </c>
       <c r="C21" s="81" t="s">
@@ -7902,9 +7908,9 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-      <c r="W21" s="22" t="str">
-        <f t="shared" ca="1" si="4"/>
-        <v/>
+      <c r="W21" s="22">
+        <f t="shared" ca="1" si="4"/>
+        <v>2</v>
       </c>
       <c r="X21" s="22" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -8176,9 +8182,9 @@
         <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
-      <c r="AD22" s="22" t="str">
-        <f t="shared" ca="1" si="5"/>
-        <v/>
+      <c r="AD22" s="22">
+        <f t="shared" ca="1" si="5"/>
+        <v>1</v>
       </c>
       <c r="AE22" s="22" t="str">
         <f t="shared" ca="1" si="5"/>
@@ -8565,7 +8571,7 @@
         <v>56</v>
       </c>
       <c r="E24" s="54">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F24" s="55">
         <v>46099</v>
@@ -8658,9 +8664,9 @@
         <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
-      <c r="AD24" s="22" t="str">
-        <f t="shared" ca="1" si="5"/>
-        <v/>
+      <c r="AD24" s="22">
+        <f t="shared" ca="1" si="5"/>
+        <v>2</v>
       </c>
       <c r="AE24" s="22" t="str">
         <f t="shared" ca="1" si="5"/>
@@ -8801,7 +8807,7 @@
     </row>
     <row r="25" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="9"/>
-      <c r="B25" s="143" t="s">
+      <c r="B25" s="126" t="s">
         <v>75</v>
       </c>
       <c r="C25" s="53" t="s">
@@ -8904,9 +8910,9 @@
         <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
-      <c r="AD25" s="22" t="str">
-        <f t="shared" ca="1" si="5"/>
-        <v/>
+      <c r="AD25" s="22">
+        <f t="shared" ca="1" si="5"/>
+        <v>2</v>
       </c>
       <c r="AE25" s="22" t="str">
         <f t="shared" ca="1" si="5"/>
@@ -9047,7 +9053,7 @@
     </row>
     <row r="26" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="9"/>
-      <c r="B26" s="144" t="s">
+      <c r="B26" s="127" t="s">
         <v>79</v>
       </c>
       <c r="C26" s="53" t="s">
@@ -9293,7 +9299,7 @@
     </row>
     <row r="27" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="9"/>
-      <c r="B27" s="143" t="s">
+      <c r="B27" s="126" t="s">
         <v>76</v>
       </c>
       <c r="C27" s="53" t="s">
@@ -9328,9 +9334,9 @@
         <f t="shared" ca="1" si="8"/>
         <v/>
       </c>
-      <c r="M27" s="22">
+      <c r="M27" s="22" t="str">
         <f t="shared" ca="1" si="8"/>
-        <v>2</v>
+        <v/>
       </c>
       <c r="N27" s="22" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -9424,9 +9430,9 @@
         <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
-      <c r="AK27" s="22" t="str">
-        <f t="shared" ca="1" si="11"/>
-        <v/>
+      <c r="AK27" s="22">
+        <f t="shared" ca="1" si="11"/>
+        <v>2</v>
       </c>
       <c r="AL27" s="22" t="str">
         <f t="shared" ca="1" si="11"/>
@@ -9546,7 +9552,7 @@
         <v>16</v>
       </c>
       <c r="D28" s="81" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="E28" s="54">
         <v>1</v>
@@ -9792,7 +9798,7 @@
         <v>16</v>
       </c>
       <c r="D29" s="81" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="E29" s="54">
         <v>1</v>
@@ -10031,7 +10037,7 @@
     </row>
     <row r="30" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="9"/>
-      <c r="B30" s="143" t="s">
+      <c r="B30" s="126" t="s">
         <v>77</v>
       </c>
       <c r="C30" s="53" t="s">
@@ -10094,105 +10100,105 @@
         <f t="shared" ca="1" si="12"/>
         <v/>
       </c>
-      <c r="T30" s="22">
-        <f t="shared" ca="1" si="12"/>
+      <c r="T30" s="22" t="str">
+        <f t="shared" ca="1" si="12"/>
+        <v/>
+      </c>
+      <c r="U30" s="22" t="str">
+        <f t="shared" ca="1" si="12"/>
+        <v/>
+      </c>
+      <c r="V30" s="22" t="str">
+        <f t="shared" ca="1" si="12"/>
+        <v/>
+      </c>
+      <c r="W30" s="22" t="str">
+        <f t="shared" ca="1" si="12"/>
+        <v/>
+      </c>
+      <c r="X30" s="22" t="str">
+        <f t="shared" ca="1" si="12"/>
+        <v/>
+      </c>
+      <c r="Y30" s="22" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+      <c r="Z30" s="22" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+      <c r="AA30" s="22" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+      <c r="AB30" s="22" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+      <c r="AC30" s="22" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+      <c r="AD30" s="22" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+      <c r="AE30" s="22" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+      <c r="AF30" s="22" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+      <c r="AG30" s="22" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+      <c r="AH30" s="22" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+      <c r="AI30" s="22" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+      <c r="AJ30" s="22" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+      <c r="AK30" s="22" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+      <c r="AL30" s="22" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+      <c r="AM30" s="22" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+      <c r="AN30" s="22" t="str">
+        <f t="shared" ca="1" si="9"/>
+        <v/>
+      </c>
+      <c r="AO30" s="22" t="str">
+        <f t="shared" ca="1" si="9"/>
+        <v/>
+      </c>
+      <c r="AP30" s="22" t="str">
+        <f t="shared" ca="1" si="9"/>
+        <v/>
+      </c>
+      <c r="AQ30" s="22" t="str">
+        <f t="shared" ca="1" si="9"/>
+        <v/>
+      </c>
+      <c r="AR30" s="22">
+        <f t="shared" ca="1" si="9"/>
         <v>2</v>
-      </c>
-      <c r="U30" s="22" t="str">
-        <f t="shared" ca="1" si="12"/>
-        <v/>
-      </c>
-      <c r="V30" s="22" t="str">
-        <f t="shared" ca="1" si="12"/>
-        <v/>
-      </c>
-      <c r="W30" s="22" t="str">
-        <f t="shared" ca="1" si="12"/>
-        <v/>
-      </c>
-      <c r="X30" s="22" t="str">
-        <f t="shared" ca="1" si="12"/>
-        <v/>
-      </c>
-      <c r="Y30" s="22" t="str">
-        <f t="shared" ca="1" si="11"/>
-        <v/>
-      </c>
-      <c r="Z30" s="22" t="str">
-        <f t="shared" ca="1" si="11"/>
-        <v/>
-      </c>
-      <c r="AA30" s="22" t="str">
-        <f t="shared" ca="1" si="11"/>
-        <v/>
-      </c>
-      <c r="AB30" s="22" t="str">
-        <f t="shared" ca="1" si="11"/>
-        <v/>
-      </c>
-      <c r="AC30" s="22" t="str">
-        <f t="shared" ca="1" si="11"/>
-        <v/>
-      </c>
-      <c r="AD30" s="22" t="str">
-        <f t="shared" ca="1" si="11"/>
-        <v/>
-      </c>
-      <c r="AE30" s="22" t="str">
-        <f t="shared" ca="1" si="11"/>
-        <v/>
-      </c>
-      <c r="AF30" s="22" t="str">
-        <f t="shared" ca="1" si="11"/>
-        <v/>
-      </c>
-      <c r="AG30" s="22" t="str">
-        <f t="shared" ca="1" si="11"/>
-        <v/>
-      </c>
-      <c r="AH30" s="22" t="str">
-        <f t="shared" ca="1" si="11"/>
-        <v/>
-      </c>
-      <c r="AI30" s="22" t="str">
-        <f t="shared" ca="1" si="11"/>
-        <v/>
-      </c>
-      <c r="AJ30" s="22" t="str">
-        <f t="shared" ca="1" si="11"/>
-        <v/>
-      </c>
-      <c r="AK30" s="22" t="str">
-        <f t="shared" ca="1" si="11"/>
-        <v/>
-      </c>
-      <c r="AL30" s="22" t="str">
-        <f t="shared" ca="1" si="11"/>
-        <v/>
-      </c>
-      <c r="AM30" s="22" t="str">
-        <f t="shared" ca="1" si="11"/>
-        <v/>
-      </c>
-      <c r="AN30" s="22" t="str">
-        <f t="shared" ca="1" si="9"/>
-        <v/>
-      </c>
-      <c r="AO30" s="22" t="str">
-        <f t="shared" ca="1" si="9"/>
-        <v/>
-      </c>
-      <c r="AP30" s="22" t="str">
-        <f t="shared" ca="1" si="9"/>
-        <v/>
-      </c>
-      <c r="AQ30" s="22" t="str">
-        <f t="shared" ca="1" si="9"/>
-        <v/>
-      </c>
-      <c r="AR30" s="22" t="str">
-        <f t="shared" ca="1" si="9"/>
-        <v/>
       </c>
       <c r="AS30" s="22" t="str">
         <f t="shared" ca="1" si="9"/>
@@ -10277,7 +10283,7 @@
     </row>
     <row r="31" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="9"/>
-      <c r="B31" s="145" t="s">
+      <c r="B31" s="128" t="s">
         <v>81</v>
       </c>
       <c r="C31" s="53"/>
@@ -10521,7 +10527,7 @@
     </row>
     <row r="32" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="9"/>
-      <c r="B32" s="142" t="s">
+      <c r="B32" s="125" t="s">
         <v>78</v>
       </c>
       <c r="C32" s="81" t="s">
@@ -10668,9 +10674,9 @@
         <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
-      <c r="AO32" s="22">
-        <f t="shared" ca="1" si="9"/>
-        <v>2</v>
+      <c r="AO32" s="22" t="str">
+        <f t="shared" ca="1" si="9"/>
+        <v/>
       </c>
       <c r="AP32" s="22" t="str">
         <f t="shared" ca="1" si="9"/>
@@ -10771,13 +10777,13 @@
         <v>69</v>
       </c>
       <c r="C33" s="81" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D33" s="81" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="E33" s="54">
-        <v>0.99</v>
+        <v>1</v>
       </c>
       <c r="F33" s="55">
         <v>46134</v>
@@ -11017,13 +11023,13 @@
         <v>66</v>
       </c>
       <c r="C34" s="81" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D34" s="81" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="E34" s="54">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F34" s="55">
         <v>46134</v>
@@ -11263,19 +11269,19 @@
         <v>62</v>
       </c>
       <c r="C35" s="53" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D35" s="53" t="s">
         <v>56</v>
       </c>
       <c r="E35" s="54">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F35" s="55">
         <v>46134</v>
       </c>
       <c r="G35" s="56">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H35" s="53"/>
       <c r="I35" s="22"/>
@@ -11341,17 +11347,19 @@
         <v>67</v>
       </c>
       <c r="C36" s="53" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D36" s="53" t="s">
         <v>56</v>
       </c>
-      <c r="E36" s="54"/>
+      <c r="E36" s="54">
+        <v>1</v>
+      </c>
       <c r="F36" s="55">
         <v>46134</v>
       </c>
       <c r="G36" s="56">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H36" s="53"/>
       <c r="I36" s="22"/>
@@ -11413,314 +11421,538 @@
     </row>
     <row r="37" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="9"/>
-      <c r="B37" s="57"/>
-      <c r="C37" s="53"/>
-      <c r="D37" s="53"/>
-      <c r="E37" s="54"/>
-      <c r="F37" s="55"/>
-      <c r="G37" s="56"/>
+      <c r="B37" s="127" t="s">
+        <v>68</v>
+      </c>
+      <c r="C37" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="D37" s="53" t="s">
+        <v>56</v>
+      </c>
+      <c r="E37" s="54">
+        <v>1</v>
+      </c>
+      <c r="F37" s="55">
+        <v>46134</v>
+      </c>
+      <c r="G37" s="56">
+        <v>8</v>
+      </c>
       <c r="H37" s="53"/>
-      <c r="I37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",I$7&gt;=$F37,I$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",I$7&gt;=$F37,I$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="J37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",J$7&gt;=$F37,J$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",J$7&gt;=$F37,J$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="K37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",K$7&gt;=$F37,K$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",K$7&gt;=$F37,K$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="L37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",L$7&gt;=$F37,L$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",L$7&gt;=$F37,L$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="M37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",M$7&gt;=$F37,M$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",M$7&gt;=$F37,M$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="N37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",N$7&gt;=$F37,N$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",N$7&gt;=$F37,N$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="O37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",O$7&gt;=$F37,O$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",O$7&gt;=$F37,O$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="P37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",P$7&gt;=$F37,P$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",P$7&gt;=$F37,P$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="Q37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",Q$7&gt;=$F37,Q$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",Q$7&gt;=$F37,Q$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="R37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",R$7&gt;=$F37,R$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",R$7&gt;=$F37,R$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="S37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",S$7&gt;=$F37,S$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",S$7&gt;=$F37,S$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="T37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",T$7&gt;=$F37,T$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",T$7&gt;=$F37,T$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="U37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",U$7&gt;=$F37,U$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",U$7&gt;=$F37,U$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="V37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",V$7&gt;=$F37,V$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",V$7&gt;=$F37,V$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="W37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",W$7&gt;=$F37,W$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",W$7&gt;=$F37,W$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="X37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",X$7&gt;=$F37,X$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",X$7&gt;=$F37,X$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="Y37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",Y$7&gt;=$F37,Y$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",Y$7&gt;=$F37,Y$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="Z37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",Z$7&gt;=$F37,Z$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",Z$7&gt;=$F37,Z$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="AA37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",AA$7&gt;=$F37,AA$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",AA$7&gt;=$F37,AA$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="AB37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",AB$7&gt;=$F37,AB$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",AB$7&gt;=$F37,AB$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="AC37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",AC$7&gt;=$F37,AC$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",AC$7&gt;=$F37,AC$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="AD37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",AD$7&gt;=$F37,AD$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",AD$7&gt;=$F37,AD$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="AE37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",AE$7&gt;=$F37,AE$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",AE$7&gt;=$F37,AE$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="AF37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",AF$7&gt;=$F37,AF$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",AF$7&gt;=$F37,AF$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="AG37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",AG$7&gt;=$F37,AG$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",AG$7&gt;=$F37,AG$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="AH37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",AH$7&gt;=$F37,AH$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",AH$7&gt;=$F37,AH$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="AI37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",AI$7&gt;=$F37,AI$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",AI$7&gt;=$F37,AI$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="AJ37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",AJ$7&gt;=$F37,AJ$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",AJ$7&gt;=$F37,AJ$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="AK37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",AK$7&gt;=$F37,AK$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",AK$7&gt;=$F37,AK$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="AL37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",AL$7&gt;=$F37,AL$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",AL$7&gt;=$F37,AL$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="AM37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",AM$7&gt;=$F37,AM$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",AM$7&gt;=$F37,AM$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="AN37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",AN$7&gt;=$F37,AN$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",AN$7&gt;=$F37,AN$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="AO37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",AO$7&gt;=$F37,AO$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",AO$7&gt;=$F37,AO$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="AP37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",AP$7&gt;=$F37,AP$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",AP$7&gt;=$F37,AP$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="AQ37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",AQ$7&gt;=$F37,AQ$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",AQ$7&gt;=$F37,AQ$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="AR37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",AR$7&gt;=$F37,AR$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",AR$7&gt;=$F37,AR$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="AS37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",AS$7&gt;=$F37,AS$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",AS$7&gt;=$F37,AS$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="AT37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",AT$7&gt;=$F37,AT$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",AT$7&gt;=$F37,AT$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="AU37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",AU$7&gt;=$F37,AU$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",AU$7&gt;=$F37,AU$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="AV37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",AV$7&gt;=$F37,AV$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",AV$7&gt;=$F37,AV$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="AW37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",AW$7&gt;=$F37,AW$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",AW$7&gt;=$F37,AW$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="AX37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",AX$7&gt;=$F37,AX$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",AX$7&gt;=$F37,AX$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="AY37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",AY$7&gt;=$F37,AY$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",AY$7&gt;=$F37,AY$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="AZ37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",AZ$7&gt;=$F37,AZ$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",AZ$7&gt;=$F37,AZ$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="BA37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",BA$7&gt;=$F37,BA$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",BA$7&gt;=$F37,BA$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="BB37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",BB$7&gt;=$F37,BB$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",BB$7&gt;=$F37,BB$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="BC37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",BC$7&gt;=$F37,BC$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",BC$7&gt;=$F37,BC$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="BD37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",BD$7&gt;=$F37,BD$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",BD$7&gt;=$F37,BD$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="BE37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",BE$7&gt;=$F37,BE$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",BE$7&gt;=$F37,BE$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="BF37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",BF$7&gt;=$F37,BF$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",BF$7&gt;=$F37,BF$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="BG37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",BG$7&gt;=$F37,BG$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",BG$7&gt;=$F37,BG$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="BH37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",BH$7&gt;=$F37,BH$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",BH$7&gt;=$F37,BH$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="BI37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",BI$7&gt;=$F37,BI$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",BI$7&gt;=$F37,BI$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="BJ37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",BJ$7&gt;=$F37,BJ$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",BJ$7&gt;=$F37,BJ$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="BK37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",BK$7&gt;=$F37,BK$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",BK$7&gt;=$F37,BK$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="BL37" s="22" t="str">
-        <f ca="1">IF(AND($C37="Goal",BL$7&gt;=$F37,BL$7&lt;=$F37+$G37-1),2,IF(AND($C37="Milestone",BL$7&gt;=$F37,BL$7&lt;=$F37+$G37-1),1,""))</f>
-        <v/>
-      </c>
-      <c r="BM37" s="83"/>
+      <c r="I37" s="22"/>
+      <c r="J37" s="22"/>
+      <c r="K37" s="22"/>
+      <c r="L37" s="22"/>
+      <c r="M37" s="22"/>
+      <c r="N37" s="22"/>
+      <c r="O37" s="22"/>
+      <c r="P37" s="22"/>
+      <c r="Q37" s="22"/>
+      <c r="R37" s="22"/>
+      <c r="S37" s="22"/>
+      <c r="T37" s="22"/>
+      <c r="U37" s="22"/>
+      <c r="V37" s="22"/>
+      <c r="W37" s="22"/>
+      <c r="X37" s="22"/>
+      <c r="Y37" s="22"/>
+      <c r="Z37" s="22"/>
+      <c r="AA37" s="22"/>
+      <c r="AB37" s="22"/>
+      <c r="AC37" s="22"/>
+      <c r="AD37" s="22"/>
+      <c r="AE37" s="22"/>
+      <c r="AF37" s="22"/>
+      <c r="AG37" s="22"/>
+      <c r="AH37" s="22"/>
+      <c r="AI37" s="22"/>
+      <c r="AJ37" s="22"/>
+      <c r="AK37" s="22"/>
+      <c r="AL37" s="22"/>
+      <c r="AM37" s="22"/>
+      <c r="AN37" s="22"/>
+      <c r="AO37" s="22"/>
+      <c r="AP37" s="22"/>
+      <c r="AQ37" s="22"/>
+      <c r="AR37" s="22"/>
+      <c r="AS37" s="22"/>
+      <c r="AT37" s="22"/>
+      <c r="AU37" s="22"/>
+      <c r="AV37" s="22"/>
+      <c r="AW37" s="22"/>
+      <c r="AX37" s="22"/>
+      <c r="AY37" s="22"/>
+      <c r="AZ37" s="22"/>
+      <c r="BA37" s="22"/>
+      <c r="BB37" s="22"/>
+      <c r="BC37" s="22"/>
+      <c r="BD37" s="22"/>
+      <c r="BE37" s="22"/>
+      <c r="BF37" s="22"/>
+      <c r="BG37" s="22"/>
+      <c r="BH37" s="22"/>
+      <c r="BI37" s="22"/>
+      <c r="BJ37" s="22"/>
+      <c r="BK37" s="22"/>
+      <c r="BL37" s="22"/>
     </row>
     <row r="38" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="10"/>
-      <c r="B38" s="111" t="s">
+      <c r="A38" s="9"/>
+      <c r="B38" s="127" t="s">
+        <v>82</v>
+      </c>
+      <c r="C38" s="53" t="s">
+        <v>9</v>
+      </c>
+      <c r="D38" s="53" t="s">
+        <v>56</v>
+      </c>
+      <c r="E38" s="54">
+        <v>1</v>
+      </c>
+      <c r="F38" s="55">
+        <v>46141</v>
+      </c>
+      <c r="G38" s="56">
+        <v>1</v>
+      </c>
+      <c r="H38" s="53"/>
+      <c r="I38" s="22"/>
+      <c r="J38" s="22"/>
+      <c r="K38" s="22"/>
+      <c r="L38" s="22"/>
+      <c r="M38" s="22"/>
+      <c r="N38" s="22"/>
+      <c r="O38" s="22"/>
+      <c r="P38" s="22"/>
+      <c r="Q38" s="22"/>
+      <c r="R38" s="22"/>
+      <c r="S38" s="22"/>
+      <c r="T38" s="22"/>
+      <c r="U38" s="22"/>
+      <c r="V38" s="22"/>
+      <c r="W38" s="22"/>
+      <c r="X38" s="22"/>
+      <c r="Y38" s="22"/>
+      <c r="Z38" s="22"/>
+      <c r="AA38" s="22"/>
+      <c r="AB38" s="22"/>
+      <c r="AC38" s="22"/>
+      <c r="AD38" s="22"/>
+      <c r="AE38" s="22"/>
+      <c r="AF38" s="22"/>
+      <c r="AG38" s="22"/>
+      <c r="AH38" s="22"/>
+      <c r="AI38" s="22"/>
+      <c r="AJ38" s="22"/>
+      <c r="AK38" s="22"/>
+      <c r="AL38" s="22"/>
+      <c r="AM38" s="22"/>
+      <c r="AN38" s="22"/>
+      <c r="AO38" s="22"/>
+      <c r="AP38" s="22"/>
+      <c r="AQ38" s="22"/>
+      <c r="AR38" s="22"/>
+      <c r="AS38" s="22"/>
+      <c r="AT38" s="22"/>
+      <c r="AU38" s="22"/>
+      <c r="AV38" s="22"/>
+      <c r="AW38" s="22"/>
+      <c r="AX38" s="22"/>
+      <c r="AY38" s="22"/>
+      <c r="AZ38" s="22"/>
+      <c r="BA38" s="22"/>
+      <c r="BB38" s="22"/>
+      <c r="BC38" s="22"/>
+      <c r="BD38" s="22"/>
+      <c r="BE38" s="22"/>
+      <c r="BF38" s="22"/>
+      <c r="BG38" s="22"/>
+      <c r="BH38" s="22"/>
+      <c r="BI38" s="22"/>
+      <c r="BJ38" s="22"/>
+      <c r="BK38" s="22"/>
+      <c r="BL38" s="22"/>
+    </row>
+    <row r="39" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="9"/>
+      <c r="B39" s="146" t="s">
+        <v>72</v>
+      </c>
+      <c r="C39" s="53"/>
+      <c r="D39" s="53"/>
+      <c r="E39" s="54"/>
+      <c r="F39" s="55"/>
+      <c r="G39" s="56"/>
+      <c r="H39" s="53"/>
+      <c r="I39" s="22"/>
+      <c r="J39" s="22"/>
+      <c r="K39" s="22"/>
+      <c r="L39" s="22"/>
+      <c r="M39" s="22"/>
+      <c r="N39" s="22"/>
+      <c r="O39" s="22"/>
+      <c r="P39" s="22"/>
+      <c r="Q39" s="22"/>
+      <c r="R39" s="22"/>
+      <c r="S39" s="22"/>
+      <c r="T39" s="22"/>
+      <c r="U39" s="22"/>
+      <c r="V39" s="22"/>
+      <c r="W39" s="22"/>
+      <c r="X39" s="22"/>
+      <c r="Y39" s="22"/>
+      <c r="Z39" s="22"/>
+      <c r="AA39" s="22"/>
+      <c r="AB39" s="22"/>
+      <c r="AC39" s="22"/>
+      <c r="AD39" s="22"/>
+      <c r="AE39" s="22"/>
+      <c r="AF39" s="22"/>
+      <c r="AG39" s="22"/>
+      <c r="AH39" s="22"/>
+      <c r="AI39" s="22"/>
+      <c r="AJ39" s="22"/>
+      <c r="AK39" s="22"/>
+      <c r="AL39" s="22"/>
+      <c r="AM39" s="22"/>
+      <c r="AN39" s="22"/>
+      <c r="AO39" s="22"/>
+      <c r="AP39" s="22"/>
+      <c r="AQ39" s="22"/>
+      <c r="AR39" s="22"/>
+      <c r="AS39" s="22"/>
+      <c r="AT39" s="22"/>
+      <c r="AU39" s="22"/>
+      <c r="AV39" s="22"/>
+      <c r="AW39" s="22"/>
+      <c r="AX39" s="22"/>
+      <c r="AY39" s="22"/>
+      <c r="AZ39" s="22"/>
+      <c r="BA39" s="22"/>
+      <c r="BB39" s="22"/>
+      <c r="BC39" s="22"/>
+      <c r="BD39" s="22"/>
+      <c r="BE39" s="22"/>
+      <c r="BF39" s="22"/>
+      <c r="BG39" s="22"/>
+      <c r="BH39" s="22"/>
+      <c r="BI39" s="22"/>
+      <c r="BJ39" s="22"/>
+      <c r="BK39" s="22"/>
+      <c r="BL39" s="22"/>
+    </row>
+    <row r="40" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="9"/>
+      <c r="B40" s="57"/>
+      <c r="C40" s="53"/>
+      <c r="D40" s="53"/>
+      <c r="E40" s="54"/>
+      <c r="F40" s="55"/>
+      <c r="G40" s="56"/>
+      <c r="H40" s="53"/>
+      <c r="I40" s="22" t="str">
+        <f t="shared" ref="I40:AN40" ca="1" si="13">IF(AND($C40="Goal",I$7&gt;=$F40,I$7&lt;=$F40+$G40-1),2,IF(AND($C40="Milestone",I$7&gt;=$F40,I$7&lt;=$F40+$G40-1),1,""))</f>
+        <v/>
+      </c>
+      <c r="J40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="K40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="L40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="M40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="N40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="O40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="P40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="Q40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="R40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="S40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="T40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="U40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="V40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="W40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="X40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="Y40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="Z40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="AA40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="AB40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="AC40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="AD40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="AE40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="AF40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="AG40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="AH40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="AI40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="AJ40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="AK40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="AL40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="AM40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="AN40" s="22" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v/>
+      </c>
+      <c r="AO40" s="22" t="str">
+        <f t="shared" ref="AO40:BL40" ca="1" si="14">IF(AND($C40="Goal",AO$7&gt;=$F40,AO$7&lt;=$F40+$G40-1),2,IF(AND($C40="Milestone",AO$7&gt;=$F40,AO$7&lt;=$F40+$G40-1),1,""))</f>
+        <v/>
+      </c>
+      <c r="AP40" s="22" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v/>
+      </c>
+      <c r="AQ40" s="22" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v/>
+      </c>
+      <c r="AR40" s="22" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v/>
+      </c>
+      <c r="AS40" s="22" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v/>
+      </c>
+      <c r="AT40" s="22" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v/>
+      </c>
+      <c r="AU40" s="22" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v/>
+      </c>
+      <c r="AV40" s="22" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v/>
+      </c>
+      <c r="AW40" s="22" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v/>
+      </c>
+      <c r="AX40" s="22" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v/>
+      </c>
+      <c r="AY40" s="22" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v/>
+      </c>
+      <c r="AZ40" s="22" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v/>
+      </c>
+      <c r="BA40" s="22" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v/>
+      </c>
+      <c r="BB40" s="22" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v/>
+      </c>
+      <c r="BC40" s="22" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v/>
+      </c>
+      <c r="BD40" s="22" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v/>
+      </c>
+      <c r="BE40" s="22" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v/>
+      </c>
+      <c r="BF40" s="22" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v/>
+      </c>
+      <c r="BG40" s="22" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v/>
+      </c>
+      <c r="BH40" s="22" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v/>
+      </c>
+      <c r="BI40" s="22" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v/>
+      </c>
+      <c r="BJ40" s="22" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v/>
+      </c>
+      <c r="BK40" s="22" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v/>
+      </c>
+      <c r="BL40" s="22" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v/>
+      </c>
+      <c r="BM40" s="83"/>
+    </row>
+    <row r="41" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="10"/>
+      <c r="B41" s="111" t="s">
         <v>20</v>
       </c>
-      <c r="C38" s="53"/>
-      <c r="D38" s="53"/>
-      <c r="E38" s="69"/>
-      <c r="F38" s="79"/>
-      <c r="G38" s="80"/>
-      <c r="H38" s="53"/>
-      <c r="I38" s="81"/>
-      <c r="J38" s="81"/>
-      <c r="K38" s="81"/>
-      <c r="L38" s="81"/>
-      <c r="M38" s="81"/>
-      <c r="N38" s="81"/>
-      <c r="O38" s="81"/>
-      <c r="P38" s="81"/>
-      <c r="Q38" s="81"/>
-      <c r="R38" s="81"/>
-      <c r="S38" s="81"/>
-      <c r="T38" s="81"/>
-      <c r="U38" s="81"/>
-      <c r="V38" s="81"/>
-      <c r="W38" s="81"/>
-      <c r="X38" s="81"/>
-      <c r="Y38" s="81"/>
-      <c r="Z38" s="81"/>
-      <c r="AA38" s="81"/>
-      <c r="AB38" s="81"/>
-      <c r="AC38" s="81"/>
-      <c r="AD38" s="81"/>
-      <c r="AE38" s="81"/>
-      <c r="AF38" s="81"/>
-      <c r="AG38" s="81"/>
-      <c r="AH38" s="81"/>
-      <c r="AI38" s="81"/>
-      <c r="AJ38" s="81"/>
-      <c r="AK38" s="81"/>
-      <c r="AL38" s="81"/>
-      <c r="AM38" s="81"/>
-      <c r="AN38" s="81"/>
-      <c r="AO38" s="81"/>
-      <c r="AP38" s="81"/>
-      <c r="AQ38" s="81"/>
-      <c r="AR38" s="81"/>
-      <c r="AS38" s="81"/>
-      <c r="AT38" s="81"/>
-      <c r="AU38" s="81"/>
-      <c r="AV38" s="81"/>
-      <c r="AW38" s="81"/>
-      <c r="AX38" s="81"/>
-      <c r="AY38" s="81"/>
-      <c r="AZ38" s="81"/>
-      <c r="BA38" s="81"/>
-      <c r="BB38" s="81"/>
-      <c r="BC38" s="81"/>
-      <c r="BD38" s="81"/>
-      <c r="BE38" s="81"/>
-      <c r="BF38" s="81"/>
-      <c r="BG38" s="81"/>
-      <c r="BH38" s="81"/>
-      <c r="BI38" s="81"/>
-      <c r="BJ38" s="81"/>
-      <c r="BK38" s="81"/>
-      <c r="BL38" s="81"/>
+      <c r="C41" s="53"/>
+      <c r="D41" s="53"/>
+      <c r="E41" s="69"/>
+      <c r="F41" s="79"/>
+      <c r="G41" s="80"/>
+      <c r="H41" s="53"/>
+      <c r="I41" s="81"/>
+      <c r="J41" s="81"/>
+      <c r="K41" s="81"/>
+      <c r="L41" s="81"/>
+      <c r="M41" s="81"/>
+      <c r="N41" s="81"/>
+      <c r="O41" s="81"/>
+      <c r="P41" s="81"/>
+      <c r="Q41" s="81"/>
+      <c r="R41" s="81"/>
+      <c r="S41" s="81"/>
+      <c r="T41" s="81"/>
+      <c r="U41" s="81"/>
+      <c r="V41" s="81"/>
+      <c r="W41" s="81"/>
+      <c r="X41" s="81"/>
+      <c r="Y41" s="81"/>
+      <c r="Z41" s="81"/>
+      <c r="AA41" s="81"/>
+      <c r="AB41" s="81"/>
+      <c r="AC41" s="81"/>
+      <c r="AD41" s="81"/>
+      <c r="AE41" s="81"/>
+      <c r="AF41" s="81"/>
+      <c r="AG41" s="81"/>
+      <c r="AH41" s="81"/>
+      <c r="AI41" s="81"/>
+      <c r="AJ41" s="81"/>
+      <c r="AK41" s="81"/>
+      <c r="AL41" s="81"/>
+      <c r="AM41" s="81"/>
+      <c r="AN41" s="81"/>
+      <c r="AO41" s="81"/>
+      <c r="AP41" s="81"/>
+      <c r="AQ41" s="81"/>
+      <c r="AR41" s="81"/>
+      <c r="AS41" s="81"/>
+      <c r="AT41" s="81"/>
+      <c r="AU41" s="81"/>
+      <c r="AV41" s="81"/>
+      <c r="AW41" s="81"/>
+      <c r="AX41" s="81"/>
+      <c r="AY41" s="81"/>
+      <c r="AZ41" s="81"/>
+      <c r="BA41" s="81"/>
+      <c r="BB41" s="81"/>
+      <c r="BC41" s="81"/>
+      <c r="BD41" s="81"/>
+      <c r="BE41" s="81"/>
+      <c r="BF41" s="81"/>
+      <c r="BG41" s="81"/>
+      <c r="BH41" s="81"/>
+      <c r="BI41" s="81"/>
+      <c r="BJ41" s="81"/>
+      <c r="BK41" s="81"/>
+      <c r="BL41" s="81"/>
     </row>
-    <row r="39" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D39" s="4"/>
-      <c r="G39" s="11"/>
-      <c r="H39" s="3"/>
+    <row r="42" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D42" s="4"/>
+      <c r="G42" s="11"/>
+      <c r="H42" s="3"/>
     </row>
-    <row r="40" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D40" s="5"/>
+    <row r="43" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D43" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -11733,7 +11965,7 @@
     <mergeCell ref="N4:Q4"/>
     <mergeCell ref="S4:V4"/>
   </mergeCells>
-  <conditionalFormatting sqref="E9:E13 E15 E17 E21 E25:E27 E30:E31 E37:E38">
+  <conditionalFormatting sqref="E9:E13 E15 E17 E21 E25:E27 E30:E31 E40:E41">
     <cfRule type="dataBar" priority="16">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -11745,60 +11977,6 @@
           <x14:id>{F10D2A26-6721-467F-A645-B5B8E195B0AB}</x14:id>
         </ext>
       </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I6:AM6">
-    <cfRule type="expression" dxfId="90" priority="15">
-      <formula>I$7&lt;=EOMONTH($I$7,0)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I6:BL6">
-    <cfRule type="expression" dxfId="89" priority="13">
-      <formula>AND(I$7&lt;=EOMONTH($I$7,1),I$7&gt;EOMONTH($I$7,0))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I7:BL38">
-    <cfRule type="expression" dxfId="88" priority="12">
-      <formula>AND(TODAY()&gt;=I$7,TODAY()&lt;J$7)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I10:BL37">
-    <cfRule type="expression" dxfId="87" priority="18" stopIfTrue="1">
-      <formula>AND($C10="Low Risk",I$7&gt;=$F10,I$7&lt;=$F10+$G10-1)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="86" priority="19" stopIfTrue="1">
-      <formula>AND($C10="High Risk",I$7&gt;=$F10,I$7&lt;=$F10+$G10-1)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="85" priority="20" stopIfTrue="1">
-      <formula>AND($C10="On Track",I$7&gt;=$F10,I$7&lt;=$F10+$G10-1)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="84" priority="21" stopIfTrue="1">
-      <formula>AND($C10="Med Risk",I$7&gt;=$F10,I$7&lt;=$F10+$G10-1)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="83" priority="22" stopIfTrue="1">
-      <formula>AND(LEN($C10)=0,I$7&gt;=$F10,I$7&lt;=$F10+$G10-1)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I38:BL38">
-    <cfRule type="expression" dxfId="82" priority="24" stopIfTrue="1">
-      <formula>AND(#REF!="Low Risk",I$7&gt;=#REF!,I$7&lt;=#REF!+#REF!-1)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="81" priority="25" stopIfTrue="1">
-      <formula>AND(#REF!="High Risk",I$7&gt;=#REF!,I$7&lt;=#REF!+#REF!-1)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="80" priority="26" stopIfTrue="1">
-      <formula>AND(#REF!="On Track",I$7&gt;=#REF!,I$7&lt;=#REF!+#REF!-1)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="79" priority="27" stopIfTrue="1">
-      <formula>AND(#REF!="Med Risk",I$7&gt;=#REF!,I$7&lt;=#REF!+#REF!-1)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="78" priority="28" stopIfTrue="1">
-      <formula>AND(LEN(#REF!)=0,I$7&gt;=#REF!,I$7&lt;=#REF!+#REF!-1)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J6:BL6">
-    <cfRule type="expression" dxfId="77" priority="14">
-      <formula>AND(J$7&lt;=EOMONTH($I$7,2),J$7&gt;EOMONTH($I$7,0),J$7&gt;EOMONTH($I$7,1))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E14">
@@ -11927,7 +12105,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E36">
+  <conditionalFormatting sqref="E36:E39">
     <cfRule type="dataBar" priority="1">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -11941,11 +12119,65 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="I6:AM6">
+    <cfRule type="expression" dxfId="90" priority="15">
+      <formula>I$7&lt;=EOMONTH($I$7,0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I6:BL6">
+    <cfRule type="expression" dxfId="89" priority="13">
+      <formula>AND(I$7&lt;=EOMONTH($I$7,1),I$7&gt;EOMONTH($I$7,0))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I7:BL41">
+    <cfRule type="expression" dxfId="88" priority="12">
+      <formula>AND(TODAY()&gt;=I$7,TODAY()&lt;J$7)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I41:BL41">
+    <cfRule type="expression" dxfId="87" priority="24" stopIfTrue="1">
+      <formula>AND(#REF!="Low Risk",I$7&gt;=#REF!,I$7&lt;=#REF!+#REF!-1)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="86" priority="25" stopIfTrue="1">
+      <formula>AND(#REF!="High Risk",I$7&gt;=#REF!,I$7&lt;=#REF!+#REF!-1)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="85" priority="26" stopIfTrue="1">
+      <formula>AND(#REF!="On Track",I$7&gt;=#REF!,I$7&lt;=#REF!+#REF!-1)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="84" priority="27" stopIfTrue="1">
+      <formula>AND(#REF!="Med Risk",I$7&gt;=#REF!,I$7&lt;=#REF!+#REF!-1)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="83" priority="28" stopIfTrue="1">
+      <formula>AND(LEN(#REF!)=0,I$7&gt;=#REF!,I$7&lt;=#REF!+#REF!-1)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J6:BL6">
+    <cfRule type="expression" dxfId="82" priority="14">
+      <formula>AND(J$7&lt;=EOMONTH($I$7,2),J$7&gt;EOMONTH($I$7,0),J$7&gt;EOMONTH($I$7,1))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I10:BL40">
+    <cfRule type="expression" dxfId="81" priority="110" stopIfTrue="1">
+      <formula>AND($C10="Low Risk",I$7&gt;=$F10,I$7&lt;=$F10+$G10-1)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="80" priority="111" stopIfTrue="1">
+      <formula>AND($C10="High Risk",I$7&gt;=$F10,I$7&lt;=$F10+$G10-1)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="79" priority="112" stopIfTrue="1">
+      <formula>AND($C10="On Track",I$7&gt;=$F10,I$7&lt;=$F10+$G10-1)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="78" priority="113" stopIfTrue="1">
+      <formula>AND($C10="Med Risk",I$7&gt;=$F10,I$7&lt;=$F10+$G10-1)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="77" priority="114" stopIfTrue="1">
+      <formula>AND(LEN($C10)=0,I$7&gt;=$F10,I$7&lt;=$F10+$G10-1)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="13">
     <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" promptTitle="Scrolling Increment" prompt="Changing this number will scroll the Gantt Chart view." sqref="C7" xr:uid="{36BE1844-BE6D-4781-8CC1-3726CFEF5A1B}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C10 C12:C37" xr:uid="{F5FB9DE8-F94E-4751-A43E-A2038BC34E10}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C10 C12:C40" xr:uid="{F5FB9DE8-F94E-4751-A43E-A2038BC34E10}">
       <formula1>"Goal,Milestone,On Track, Low Risk, Med Risk, High Risk"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" sqref="C11" xr:uid="{F40D2BC0-4DE6-4E46-B927-0ABBD58CC55D}">
@@ -11959,12 +12191,12 @@
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="A scrollbar is in cells I8 through BL8. _x000a_To jump forward or backward in the timeline, enter a value of 0 or higher in cell C7._x000a_A value of 0 takes you to the beginning of the chart." sqref="A8" xr:uid="{20BDAE11-8D94-4CD5-9BB5-4ED61ECE0339}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="This row contains headers for the project schedule.  B9 through G9 contains schedule information.  Cells I9 through BL9 contain the first letter of each day of the week for the date above that heading._x000a_All project timeline charting is auto generated." sqref="A9" xr:uid="{2FF2EDD9-EF71-4F8A-AEC1-573F570081A3}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Project information starting in cell B11 through cell G11. _x000a_Enter Milestone Description, select a Category, assign someone to the task, and enter the progress, start date, and number of days for the task to start charting._x000a_" sqref="A11" xr:uid="{F0E8EBCB-B90E-4A0B-8C81-7F34870BDCA1}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="This row marks the end of the Gantt milestone data. DO NOT enter anything in this row. _x000a_To add more items, insert new rows above this one._x000a_" sqref="A38" xr:uid="{924AD4A5-6654-46D8-A99A-F39984BDA1A9}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="This is an empty row" sqref="A37" xr:uid="{4769C95E-0C34-4BFE-AD69-266D3B34DDAE}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="This row marks the end of the Gantt milestone data. DO NOT enter anything in this row. _x000a_To add more items, insert new rows above this one._x000a_" sqref="A41" xr:uid="{924AD4A5-6654-46D8-A99A-F39984BDA1A9}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="This is an empty row" sqref="A40" xr:uid="{4769C95E-0C34-4BFE-AD69-266D3B34DDAE}"/>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
-  <pageSetup scale="45" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageSetup scale="40" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <headerFooter differentFirst="1" scaleWithDoc="0">
     <oddFooter>Page &amp;P of &amp;N</oddFooter>
   </headerFooter>
@@ -12017,45 +12249,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>E9:E13 E15 E17 E21 E25:E27 E30:E31 E37:E38</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="iconSet" priority="17" id="{36318585-8B22-4FB7-8876-1BFC78FE3731}">
-            <x14:iconSet iconSet="3Stars" showValue="0" custom="1">
-              <x14:cfvo type="percent">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>1</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:cfIcon iconSet="NoIcons" iconId="0"/>
-              <x14:cfIcon iconSet="3Flags" iconId="1"/>
-              <x14:cfIcon iconSet="3Signs" iconId="0"/>
-            </x14:iconSet>
-          </x14:cfRule>
-          <xm:sqref>I10:BL37</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="iconSet" priority="23" id="{B61B6C73-D19B-48D0-9C8D-40E9A01FF0D4}">
-            <x14:iconSet iconSet="3Stars" showValue="0" custom="1">
-              <x14:cfvo type="percent">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>1</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:cfIcon iconSet="NoIcons" iconId="0"/>
-              <x14:cfIcon iconSet="3Flags" iconId="1"/>
-              <x14:cfIcon iconSet="3Signs" iconId="0"/>
-            </x14:iconSet>
-          </x14:cfRule>
-          <xm:sqref>I38:BL38</xm:sqref>
+          <xm:sqref>E9:E13 E15 E17 E21 E25:E27 E30:E31 E40:E41</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{E11DE259-0E26-4176-8A37-397989E52933}">
@@ -12205,7 +12399,45 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>E36</xm:sqref>
+          <xm:sqref>E36:E39</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="iconSet" priority="23" id="{B61B6C73-D19B-48D0-9C8D-40E9A01FF0D4}">
+            <x14:iconSet iconSet="3Stars" showValue="0" custom="1">
+              <x14:cfvo type="percent">
+                <xm:f>0</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="num">
+                <xm:f>1</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="num">
+                <xm:f>2</xm:f>
+              </x14:cfvo>
+              <x14:cfIcon iconSet="NoIcons" iconId="0"/>
+              <x14:cfIcon iconSet="3Flags" iconId="1"/>
+              <x14:cfIcon iconSet="3Signs" iconId="0"/>
+            </x14:iconSet>
+          </x14:cfRule>
+          <xm:sqref>I41:BL41</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="iconSet" priority="109" id="{36318585-8B22-4FB7-8876-1BFC78FE3731}">
+            <x14:iconSet iconSet="3Stars" showValue="0" custom="1">
+              <x14:cfvo type="percent">
+                <xm:f>0</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="num">
+                <xm:f>1</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="num">
+                <xm:f>2</xm:f>
+              </x14:cfvo>
+              <x14:cfIcon iconSet="NoIcons" iconId="0"/>
+              <x14:cfIcon iconSet="3Flags" iconId="1"/>
+              <x14:cfIcon iconSet="3Signs" iconId="0"/>
+            </x14:iconSet>
+          </x14:cfRule>
+          <xm:sqref>I10:BL40</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -12236,27 +12468,27 @@
     <row r="1" spans="1:68" ht="25.15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="1:68" ht="49.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="10"/>
-      <c r="B2" s="127" t="s">
+      <c r="B2" s="131" t="s">
         <v>73</v>
       </c>
-      <c r="C2" s="127"/>
-      <c r="D2" s="127"/>
-      <c r="E2" s="127"/>
-      <c r="F2" s="127"/>
-      <c r="G2" s="127"/>
-      <c r="H2" s="127"/>
-      <c r="I2" s="128"/>
-      <c r="J2" s="128"/>
-      <c r="K2" s="128"/>
-      <c r="L2" s="128"/>
-      <c r="M2" s="128"/>
-      <c r="N2" s="128"/>
-      <c r="O2" s="129"/>
-      <c r="P2" s="129"/>
-      <c r="Q2" s="129"/>
-      <c r="R2" s="129"/>
-      <c r="S2" s="129"/>
-      <c r="T2" s="129"/>
+      <c r="C2" s="131"/>
+      <c r="D2" s="131"/>
+      <c r="E2" s="131"/>
+      <c r="F2" s="131"/>
+      <c r="G2" s="131"/>
+      <c r="H2" s="131"/>
+      <c r="I2" s="132"/>
+      <c r="J2" s="132"/>
+      <c r="K2" s="132"/>
+      <c r="L2" s="132"/>
+      <c r="M2" s="132"/>
+      <c r="N2" s="132"/>
+      <c r="O2" s="133"/>
+      <c r="P2" s="133"/>
+      <c r="Q2" s="133"/>
+      <c r="R2" s="133"/>
+      <c r="S2" s="133"/>
+      <c r="T2" s="133"/>
       <c r="U2" s="61"/>
       <c r="V2" s="61"/>
       <c r="W2" s="61"/>
@@ -12330,36 +12562,36 @@
         <v>18</v>
       </c>
       <c r="H4" s="69"/>
-      <c r="I4" s="130" t="s">
+      <c r="I4" s="134" t="s">
         <v>25</v>
       </c>
-      <c r="J4" s="130"/>
-      <c r="K4" s="130"/>
-      <c r="L4" s="130"/>
-      <c r="N4" s="131" t="s">
+      <c r="J4" s="134"/>
+      <c r="K4" s="134"/>
+      <c r="L4" s="134"/>
+      <c r="N4" s="135" t="s">
         <v>26</v>
       </c>
-      <c r="O4" s="131"/>
-      <c r="P4" s="131"/>
-      <c r="Q4" s="131"/>
-      <c r="S4" s="132" t="s">
+      <c r="O4" s="135"/>
+      <c r="P4" s="135"/>
+      <c r="Q4" s="135"/>
+      <c r="S4" s="136" t="s">
         <v>27</v>
       </c>
-      <c r="T4" s="132"/>
-      <c r="U4" s="132"/>
-      <c r="V4" s="132"/>
-      <c r="X4" s="125" t="s">
+      <c r="T4" s="136"/>
+      <c r="U4" s="136"/>
+      <c r="V4" s="136"/>
+      <c r="X4" s="129" t="s">
         <v>28</v>
       </c>
-      <c r="Y4" s="125"/>
-      <c r="Z4" s="125"/>
-      <c r="AA4" s="125"/>
-      <c r="AC4" s="126" t="s">
+      <c r="Y4" s="129"/>
+      <c r="Z4" s="129"/>
+      <c r="AA4" s="129"/>
+      <c r="AC4" s="130" t="s">
         <v>19</v>
       </c>
-      <c r="AD4" s="126"/>
-      <c r="AE4" s="126"/>
-      <c r="AF4" s="126"/>
+      <c r="AD4" s="130"/>
+      <c r="AE4" s="130"/>
+      <c r="AF4" s="130"/>
     </row>
     <row r="5" spans="1:68" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="10"/>
@@ -19446,27 +19678,27 @@
     <row r="1" spans="1:68" ht="25.15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="1:68" ht="49.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="10"/>
-      <c r="B2" s="127" t="s">
+      <c r="B2" s="131" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="127"/>
-      <c r="D2" s="127"/>
-      <c r="E2" s="127"/>
-      <c r="F2" s="127"/>
-      <c r="G2" s="127"/>
-      <c r="H2" s="127"/>
-      <c r="I2" s="128"/>
-      <c r="J2" s="128"/>
-      <c r="K2" s="128"/>
-      <c r="L2" s="128"/>
-      <c r="M2" s="128"/>
-      <c r="N2" s="128"/>
-      <c r="O2" s="129"/>
-      <c r="P2" s="129"/>
-      <c r="Q2" s="129"/>
-      <c r="R2" s="129"/>
-      <c r="S2" s="129"/>
-      <c r="T2" s="129"/>
+      <c r="C2" s="131"/>
+      <c r="D2" s="131"/>
+      <c r="E2" s="131"/>
+      <c r="F2" s="131"/>
+      <c r="G2" s="131"/>
+      <c r="H2" s="131"/>
+      <c r="I2" s="132"/>
+      <c r="J2" s="132"/>
+      <c r="K2" s="132"/>
+      <c r="L2" s="132"/>
+      <c r="M2" s="132"/>
+      <c r="N2" s="132"/>
+      <c r="O2" s="133"/>
+      <c r="P2" s="133"/>
+      <c r="Q2" s="133"/>
+      <c r="R2" s="133"/>
+      <c r="S2" s="133"/>
+      <c r="T2" s="133"/>
       <c r="U2" s="61"/>
       <c r="V2" s="61"/>
       <c r="W2" s="61"/>
@@ -19540,36 +19772,36 @@
         <v>18</v>
       </c>
       <c r="H4" s="69"/>
-      <c r="I4" s="130" t="s">
+      <c r="I4" s="134" t="s">
         <v>25</v>
       </c>
-      <c r="J4" s="130"/>
-      <c r="K4" s="130"/>
-      <c r="L4" s="130"/>
-      <c r="N4" s="131" t="s">
+      <c r="J4" s="134"/>
+      <c r="K4" s="134"/>
+      <c r="L4" s="134"/>
+      <c r="N4" s="135" t="s">
         <v>26</v>
       </c>
-      <c r="O4" s="131"/>
-      <c r="P4" s="131"/>
-      <c r="Q4" s="131"/>
-      <c r="S4" s="132" t="s">
+      <c r="O4" s="135"/>
+      <c r="P4" s="135"/>
+      <c r="Q4" s="135"/>
+      <c r="S4" s="136" t="s">
         <v>27</v>
       </c>
-      <c r="T4" s="132"/>
-      <c r="U4" s="132"/>
-      <c r="V4" s="132"/>
-      <c r="X4" s="125" t="s">
+      <c r="T4" s="136"/>
+      <c r="U4" s="136"/>
+      <c r="V4" s="136"/>
+      <c r="X4" s="129" t="s">
         <v>28</v>
       </c>
-      <c r="Y4" s="125"/>
-      <c r="Z4" s="125"/>
-      <c r="AA4" s="125"/>
-      <c r="AC4" s="126" t="s">
+      <c r="Y4" s="129"/>
+      <c r="Z4" s="129"/>
+      <c r="AA4" s="129"/>
+      <c r="AC4" s="130" t="s">
         <v>19</v>
       </c>
-      <c r="AD4" s="126"/>
-      <c r="AE4" s="126"/>
-      <c r="AF4" s="126"/>
+      <c r="AD4" s="130"/>
+      <c r="AE4" s="130"/>
+      <c r="AF4" s="130"/>
     </row>
     <row r="5" spans="1:68" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="10"/>
@@ -26656,27 +26888,27 @@
     <row r="1" spans="1:68" ht="25.15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="1:68" ht="49.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="10"/>
-      <c r="B2" s="135" t="s">
+      <c r="B2" s="139" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="135"/>
-      <c r="D2" s="135"/>
-      <c r="E2" s="135"/>
-      <c r="F2" s="135"/>
-      <c r="G2" s="135"/>
-      <c r="H2" s="135"/>
-      <c r="I2" s="136"/>
-      <c r="J2" s="136"/>
-      <c r="K2" s="136"/>
-      <c r="L2" s="136"/>
-      <c r="M2" s="136"/>
-      <c r="N2" s="136"/>
-      <c r="O2" s="137"/>
-      <c r="P2" s="138"/>
-      <c r="Q2" s="138"/>
-      <c r="R2" s="138"/>
-      <c r="S2" s="138"/>
-      <c r="T2" s="138"/>
+      <c r="C2" s="139"/>
+      <c r="D2" s="139"/>
+      <c r="E2" s="139"/>
+      <c r="F2" s="139"/>
+      <c r="G2" s="139"/>
+      <c r="H2" s="139"/>
+      <c r="I2" s="140"/>
+      <c r="J2" s="140"/>
+      <c r="K2" s="140"/>
+      <c r="L2" s="140"/>
+      <c r="M2" s="140"/>
+      <c r="N2" s="140"/>
+      <c r="O2" s="141"/>
+      <c r="P2" s="142"/>
+      <c r="Q2" s="142"/>
+      <c r="R2" s="142"/>
+      <c r="S2" s="142"/>
+      <c r="T2" s="142"/>
       <c r="U2" s="20"/>
       <c r="V2" s="20"/>
       <c r="W2" s="20"/>
@@ -26803,40 +27035,40 @@
         <v>18</v>
       </c>
       <c r="H4" s="25"/>
-      <c r="I4" s="130" t="s">
+      <c r="I4" s="134" t="s">
         <v>25</v>
       </c>
-      <c r="J4" s="130"/>
-      <c r="K4" s="130"/>
-      <c r="L4" s="130"/>
+      <c r="J4" s="134"/>
+      <c r="K4" s="134"/>
+      <c r="L4" s="134"/>
       <c r="M4" s="28"/>
-      <c r="N4" s="131" t="s">
+      <c r="N4" s="135" t="s">
         <v>26</v>
       </c>
-      <c r="O4" s="131"/>
-      <c r="P4" s="131"/>
-      <c r="Q4" s="131"/>
+      <c r="O4" s="135"/>
+      <c r="P4" s="135"/>
+      <c r="Q4" s="135"/>
       <c r="R4" s="28"/>
-      <c r="S4" s="132" t="s">
+      <c r="S4" s="136" t="s">
         <v>27</v>
       </c>
-      <c r="T4" s="132"/>
-      <c r="U4" s="132"/>
-      <c r="V4" s="132"/>
+      <c r="T4" s="136"/>
+      <c r="U4" s="136"/>
+      <c r="V4" s="136"/>
       <c r="W4" s="28"/>
-      <c r="X4" s="125" t="s">
+      <c r="X4" s="129" t="s">
         <v>28</v>
       </c>
-      <c r="Y4" s="125"/>
-      <c r="Z4" s="125"/>
-      <c r="AA4" s="125"/>
+      <c r="Y4" s="129"/>
+      <c r="Z4" s="129"/>
+      <c r="AA4" s="129"/>
       <c r="AB4" s="28"/>
-      <c r="AC4" s="126" t="s">
+      <c r="AC4" s="130" t="s">
         <v>19</v>
       </c>
-      <c r="AD4" s="126"/>
-      <c r="AE4" s="126"/>
-      <c r="AF4" s="126"/>
+      <c r="AD4" s="130"/>
+      <c r="AE4" s="130"/>
+      <c r="AF4" s="130"/>
       <c r="AG4" s="28"/>
       <c r="AH4" s="28"/>
       <c r="AI4" s="28"/>
@@ -34316,27 +34548,27 @@
     <row r="1" spans="1:68" ht="25.15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="1:68" ht="49.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="10"/>
-      <c r="B2" s="139" t="s">
+      <c r="B2" s="143" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="139"/>
-      <c r="D2" s="139"/>
-      <c r="E2" s="139"/>
-      <c r="F2" s="139"/>
-      <c r="G2" s="139"/>
-      <c r="H2" s="139"/>
-      <c r="I2" s="140"/>
-      <c r="J2" s="140"/>
-      <c r="K2" s="140"/>
-      <c r="L2" s="140"/>
-      <c r="M2" s="140"/>
-      <c r="N2" s="140"/>
-      <c r="O2" s="141"/>
-      <c r="P2" s="141"/>
-      <c r="Q2" s="141"/>
-      <c r="R2" s="141"/>
-      <c r="S2" s="141"/>
-      <c r="T2" s="141"/>
+      <c r="C2" s="143"/>
+      <c r="D2" s="143"/>
+      <c r="E2" s="143"/>
+      <c r="F2" s="143"/>
+      <c r="G2" s="143"/>
+      <c r="H2" s="143"/>
+      <c r="I2" s="144"/>
+      <c r="J2" s="144"/>
+      <c r="K2" s="144"/>
+      <c r="L2" s="144"/>
+      <c r="M2" s="144"/>
+      <c r="N2" s="144"/>
+      <c r="O2" s="145"/>
+      <c r="P2" s="145"/>
+      <c r="Q2" s="145"/>
+      <c r="R2" s="145"/>
+      <c r="S2" s="145"/>
+      <c r="T2" s="145"/>
       <c r="U2" s="91"/>
       <c r="V2" s="91"/>
       <c r="W2" s="91"/>
@@ -34410,36 +34642,36 @@
         <v>18</v>
       </c>
       <c r="H4" s="69"/>
-      <c r="I4" s="130" t="s">
+      <c r="I4" s="134" t="s">
         <v>25</v>
       </c>
-      <c r="J4" s="130"/>
-      <c r="K4" s="130"/>
-      <c r="L4" s="130"/>
-      <c r="N4" s="131" t="s">
+      <c r="J4" s="134"/>
+      <c r="K4" s="134"/>
+      <c r="L4" s="134"/>
+      <c r="N4" s="135" t="s">
         <v>26</v>
       </c>
-      <c r="O4" s="131"/>
-      <c r="P4" s="131"/>
-      <c r="Q4" s="131"/>
-      <c r="S4" s="132" t="s">
+      <c r="O4" s="135"/>
+      <c r="P4" s="135"/>
+      <c r="Q4" s="135"/>
+      <c r="S4" s="136" t="s">
         <v>27</v>
       </c>
-      <c r="T4" s="132"/>
-      <c r="U4" s="132"/>
-      <c r="V4" s="132"/>
-      <c r="X4" s="125" t="s">
+      <c r="T4" s="136"/>
+      <c r="U4" s="136"/>
+      <c r="V4" s="136"/>
+      <c r="X4" s="129" t="s">
         <v>28</v>
       </c>
-      <c r="Y4" s="125"/>
-      <c r="Z4" s="125"/>
-      <c r="AA4" s="125"/>
-      <c r="AC4" s="126" t="s">
+      <c r="Y4" s="129"/>
+      <c r="Z4" s="129"/>
+      <c r="AA4" s="129"/>
+      <c r="AC4" s="130" t="s">
         <v>19</v>
       </c>
-      <c r="AD4" s="126"/>
-      <c r="AE4" s="126"/>
-      <c r="AF4" s="126"/>
+      <c r="AD4" s="130"/>
+      <c r="AE4" s="130"/>
+      <c r="AF4" s="130"/>
     </row>
     <row r="5" spans="1:68" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="10"/>
@@ -41492,25 +41724,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="22a266b9fa9a230c5a512669d8b298c3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="eddc33fff6b14141ee5c74a0d29ea6a1" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -41786,6 +41999,25 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Image>
+    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{39060724-9CA2-4290-8A0C-B53624A594E7}">
   <ds:schemaRefs>
@@ -41795,18 +42027,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA4BA2A8-DB97-40F9-8DB6-154C09C7467C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75C87518-DD8E-42CD-8DAC-291A323E849B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -41825,4 +42045,16 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA4BA2A8-DB97-40F9-8DB6-154C09C7467C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
+    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>